<commit_message>
Update Bm the nguoi 01.09
</commit_message>
<xml_diff>
--- a/EPORTAL/App_Data/BM_Đăng ký thẻ người.xlsx
+++ b/EPORTAL/App_Data/BM_Đăng ký thẻ người.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BaoBao\EPORTAL\EPORTAL\EPORTAL\App_Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive - hoaphat.com.vn\Software\EPORTAL_DEV\EPORTAL\EPORTAL\EPORTAL\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA36604C-2E5E-41C7-AC42-A10E431A46EA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8657FDA5-7E92-49D9-93D1-17C43CA3462E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BM" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,6 @@
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="56">
   <si>
     <t>ĐƠN ĐỀ NGHỊ CẤP LẠI/ GIA HẠN/ ĐIỀU CHỈNH THÔNG TIN THẺ NGƯỜI</t>
   </si>
@@ -109,9 +108,6 @@
     <t>Cấp lại</t>
   </si>
   <si>
-    <t>Chuyển đổi NT</t>
-  </si>
-  <si>
     <t>2. HPDQ1 -  NHÀ MÁY LUYỆN CỐC</t>
   </si>
   <si>
@@ -203,18 +199,18 @@
 (Đánh dấu "X" nếu đăng ký)"</t>
   </si>
   <si>
+    <t>CHỨC VỤ</t>
+  </si>
+  <si>
+    <t>KHU VỰC LÀM VIỆC</t>
+  </si>
+  <si>
+    <t>CỔNG ĐĂNG KÝ RA/VÀO</t>
+  </si>
+  <si>
     <t>BM.03A/QT.20
-Ngày hiệu lực: 30/11/2024
-Lần sửa đổi: 02</t>
-  </si>
-  <si>
-    <t>CHỨC VỤ</t>
-  </si>
-  <si>
-    <t>KHU VỰC LÀM VIỆC</t>
-  </si>
-  <si>
-    <t>CỔNG ĐĂNG KÝ RA/VÀO</t>
+Ngày hiệu lực: 01/09/2025
+Lần sửa đổi: 03</t>
   </si>
 </sst>
 </file>
@@ -501,63 +497,63 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -605,7 +601,7 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="2210666" cy="975880"/>
+          <a:ext cx="2205718" cy="978354"/>
           <a:chOff x="0" y="57150"/>
           <a:chExt cx="2219325" cy="981075"/>
         </a:xfrm>
@@ -993,7 +989,7 @@
     <col min="11" max="11" width="13.28515625" style="9" customWidth="1"/>
     <col min="12" max="12" width="11.7109375" style="9" customWidth="1"/>
     <col min="13" max="14" width="10" style="9" customWidth="1"/>
-    <col min="15" max="15" width="14.140625" style="9" customWidth="1"/>
+    <col min="15" max="15" width="14.140625" style="9" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="18.140625" style="10" customWidth="1"/>
     <col min="17" max="17" width="83" style="10" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="37.5703125" style="9" bestFit="1" customWidth="1"/>
@@ -1006,112 +1002,112 @@
   <sheetData>
     <row r="1" spans="1:24" s="1" customFormat="1" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C1" s="31"/>
-      <c r="K1" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="35"/>
+      <c r="K1" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+      <c r="P1" s="39"/>
+      <c r="Q1" s="39"/>
+      <c r="R1" s="39"/>
+      <c r="S1" s="39"/>
+      <c r="T1" s="39"/>
     </row>
     <row r="2" spans="1:24" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-      <c r="O2" s="36"/>
-      <c r="P2" s="36"/>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
-      <c r="T2" s="36"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
+      <c r="J2" s="40"/>
+      <c r="K2" s="40"/>
+      <c r="L2" s="40"/>
+      <c r="M2" s="40"/>
+      <c r="N2" s="40"/>
+      <c r="O2" s="40"/>
+      <c r="P2" s="40"/>
+      <c r="Q2" s="40"/>
+      <c r="R2" s="40"/>
+      <c r="S2" s="40"/>
+      <c r="T2" s="40"/>
     </row>
     <row r="3" spans="1:24" s="1" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="32"/>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="32"/>
-      <c r="L3" s="32"/>
-      <c r="M3" s="32"/>
-      <c r="N3" s="32"/>
-      <c r="O3" s="32"/>
-      <c r="P3" s="32"/>
-      <c r="Q3" s="32"/>
-      <c r="R3" s="32"/>
-      <c r="S3" s="32"/>
-      <c r="T3" s="32"/>
+      <c r="A3" s="38"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="38"/>
+      <c r="I3" s="38"/>
+      <c r="J3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="38"/>
+      <c r="M3" s="38"/>
+      <c r="N3" s="38"/>
+      <c r="O3" s="38"/>
+      <c r="P3" s="38"/>
+      <c r="Q3" s="38"/>
+      <c r="R3" s="38"/>
+      <c r="S3" s="38"/>
+      <c r="T3" s="38"/>
     </row>
     <row r="4" spans="1:24" s="1" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="C4" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="39" t="s">
+      <c r="D4" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="39" t="s">
+      <c r="E4" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="39" t="s">
+      <c r="F4" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="39" t="s">
+      <c r="G4" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="33" t="s">
+      <c r="H4" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="33" t="s">
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="L4" s="34"/>
-      <c r="M4" s="34"/>
-      <c r="N4" s="34"/>
-      <c r="O4" s="48"/>
-      <c r="P4" s="43" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q4" s="41" t="s">
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="36"/>
+      <c r="O4" s="37"/>
+      <c r="P4" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q4" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="45" t="s">
+      <c r="R4" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="S4" s="47" t="s">
+      <c r="S4" s="51" t="s">
         <v>12</v>
       </c>
-      <c r="T4" s="37" t="s">
+      <c r="T4" s="41" t="s">
         <v>13</v>
       </c>
       <c r="X4" s="2" t="s">
@@ -1119,13 +1115,13 @@
       </c>
     </row>
     <row r="5" spans="1:24" s="1" customFormat="1" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="38"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
+      <c r="A5" s="42"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
       <c r="H5" s="5" t="s">
         <v>15</v>
       </c>
@@ -1147,16 +1143,14 @@
       <c r="N5" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="O5" s="5" t="s">
+      <c r="O5" s="5"/>
+      <c r="P5" s="48"/>
+      <c r="Q5" s="46"/>
+      <c r="R5" s="50"/>
+      <c r="S5" s="51"/>
+      <c r="T5" s="42"/>
+      <c r="X5" s="4" t="s">
         <v>22</v>
-      </c>
-      <c r="P5" s="44"/>
-      <c r="Q5" s="42"/>
-      <c r="R5" s="46"/>
-      <c r="S5" s="47"/>
-      <c r="T5" s="38"/>
-      <c r="X5" s="4" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:24" s="7" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1363,6 +1357,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="S4:S5"/>
     <mergeCell ref="K4:O4"/>
     <mergeCell ref="A3:T3"/>
     <mergeCell ref="H4:J4"/>
@@ -1379,7 +1374,6 @@
     <mergeCell ref="T4:T5"/>
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="G4:G5"/>
-    <mergeCell ref="S4:S5"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <dataValidations count="1">
@@ -1409,25 +1403,25 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B1" s="14"/>
-      <c r="C1" s="49" t="s">
-        <v>55</v>
-      </c>
-      <c r="D1" s="50"/>
+      <c r="C1" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" s="33"/>
       <c r="E1" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="4"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="51"/>
-      <c r="H1" s="4" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -1437,7 +1431,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="12"/>
@@ -1447,7 +1441,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
@@ -1607,15 +1601,15 @@
   <sheetData>
     <row r="1" spans="1:2" s="3" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>14</v>
@@ -1623,128 +1617,128 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B14" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="581" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A581" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="582" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A582" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="583" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A583" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="584" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A584" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>